<commit_message>
Add STS & Jump to Tasks Report
</commit_message>
<xml_diff>
--- a/Results/Jump/Comparisons/Overall_Comparison_Jump.xlsx
+++ b/Results/Jump/Comparisons/Overall_Comparison_Jump.xlsx
@@ -10,6 +10,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All_Scenarios" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deltas_vs_Baseline" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base_vs_Pipeline_PCA" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base_vs_Detected_Action" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Base_vs_Detected_Action_Pipelin" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -427,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L7"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -742,6 +744,258 @@
       </c>
       <c r="L7" t="n">
         <v>9.708480712309099</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Detected_Action</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SVM</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>87.19999999999999</v>
+      </c>
+      <c r="D8" t="n">
+        <v>6.061414087549267</v>
+      </c>
+      <c r="E8" t="n">
+        <v>91.13756613756614</v>
+      </c>
+      <c r="F8" t="n">
+        <v>3.080015874701917</v>
+      </c>
+      <c r="G8" t="n">
+        <v>87.19999999999999</v>
+      </c>
+      <c r="H8" t="n">
+        <v>6.061414087549265</v>
+      </c>
+      <c r="I8" t="n">
+        <v>93.60000000000002</v>
+      </c>
+      <c r="J8" t="n">
+        <v>3.030707043774636</v>
+      </c>
+      <c r="K8" t="n">
+        <v>87.12161912161912</v>
+      </c>
+      <c r="L8" t="n">
+        <v>6.15826055847296</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Detected_Action</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Random Forest</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>87.2</v>
+      </c>
+      <c r="D9" t="n">
+        <v>6.917503296121502</v>
+      </c>
+      <c r="E9" t="n">
+        <v>88.70952380952382</v>
+      </c>
+      <c r="F9" t="n">
+        <v>6.566022717063021</v>
+      </c>
+      <c r="G9" t="n">
+        <v>87.2</v>
+      </c>
+      <c r="H9" t="n">
+        <v>6.917503296121498</v>
+      </c>
+      <c r="I9" t="n">
+        <v>93.59999999999999</v>
+      </c>
+      <c r="J9" t="n">
+        <v>3.458751648060752</v>
+      </c>
+      <c r="K9" t="n">
+        <v>86.92155252155253</v>
+      </c>
+      <c r="L9" t="n">
+        <v>7.18419586820018</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Detected_Action</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>KNN</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>75.2</v>
+      </c>
+      <c r="D10" t="n">
+        <v>7.822095958576909</v>
+      </c>
+      <c r="E10" t="n">
+        <v>78.41428571428571</v>
+      </c>
+      <c r="F10" t="n">
+        <v>11.76869211874737</v>
+      </c>
+      <c r="G10" t="n">
+        <v>75.2</v>
+      </c>
+      <c r="H10" t="n">
+        <v>7.82209595857691</v>
+      </c>
+      <c r="I10" t="n">
+        <v>87.59999999999999</v>
+      </c>
+      <c r="J10" t="n">
+        <v>3.911047979288451</v>
+      </c>
+      <c r="K10" t="n">
+        <v>72.51971731971732</v>
+      </c>
+      <c r="L10" t="n">
+        <v>9.950502325671245</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Detected_Action_Pipeline_PCA</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>SVM</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>92.8</v>
+      </c>
+      <c r="D11" t="n">
+        <v>5.41602560309064</v>
+      </c>
+      <c r="E11" t="n">
+        <v>94.17460317460318</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4.378167008108077</v>
+      </c>
+      <c r="G11" t="n">
+        <v>92.8</v>
+      </c>
+      <c r="H11" t="n">
+        <v>5.416025603090637</v>
+      </c>
+      <c r="I11" t="n">
+        <v>96.40000000000001</v>
+      </c>
+      <c r="J11" t="n">
+        <v>2.70801280154532</v>
+      </c>
+      <c r="K11" t="n">
+        <v>92.71717171717169</v>
+      </c>
+      <c r="L11" t="n">
+        <v>5.384251873454774</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Detected_Action_Pipeline_PCA</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Random Forest</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>84.53333333333335</v>
+      </c>
+      <c r="D12" t="n">
+        <v>7.128451081042419</v>
+      </c>
+      <c r="E12" t="n">
+        <v>86.60634920634921</v>
+      </c>
+      <c r="F12" t="n">
+        <v>7.088862276835729</v>
+      </c>
+      <c r="G12" t="n">
+        <v>84.53333333333335</v>
+      </c>
+      <c r="H12" t="n">
+        <v>7.128451081042415</v>
+      </c>
+      <c r="I12" t="n">
+        <v>92.26666666666667</v>
+      </c>
+      <c r="J12" t="n">
+        <v>3.564225540521208</v>
+      </c>
+      <c r="K12" t="n">
+        <v>84.08620268620268</v>
+      </c>
+      <c r="L12" t="n">
+        <v>7.599715627198697</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Detected_Action_Pipeline_PCA</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>KNN</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>72.26666666666667</v>
+      </c>
+      <c r="D13" t="n">
+        <v>7.620634755325445</v>
+      </c>
+      <c r="E13" t="n">
+        <v>75.06137566137566</v>
+      </c>
+      <c r="F13" t="n">
+        <v>12.2421003422925</v>
+      </c>
+      <c r="G13" t="n">
+        <v>72.26666666666667</v>
+      </c>
+      <c r="H13" t="n">
+        <v>7.620634755325447</v>
+      </c>
+      <c r="I13" t="n">
+        <v>86.13333333333334</v>
+      </c>
+      <c r="J13" t="n">
+        <v>3.810317377662719</v>
+      </c>
+      <c r="K13" t="n">
+        <v>68.8015984015984</v>
+      </c>
+      <c r="L13" t="n">
+        <v>9.810457993018462</v>
       </c>
     </row>
   </sheetData>
@@ -755,7 +1009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q4"/>
+  <dimension ref="A1:Q10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1014,6 +1268,348 @@
       </c>
       <c r="Q4" t="n">
         <v>-3.26080586080586</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Detected_Action</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SVM</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>87.19999999999999</v>
+      </c>
+      <c r="D5" t="n">
+        <v>91.13756613756614</v>
+      </c>
+      <c r="E5" t="n">
+        <v>87.19999999999999</v>
+      </c>
+      <c r="F5" t="n">
+        <v>93.60000000000002</v>
+      </c>
+      <c r="G5" t="n">
+        <v>87.12161912161912</v>
+      </c>
+      <c r="H5" t="n">
+        <v>89.59999999999998</v>
+      </c>
+      <c r="I5" t="n">
+        <v>91.96984126984125</v>
+      </c>
+      <c r="J5" t="n">
+        <v>89.59999999999999</v>
+      </c>
+      <c r="K5" t="n">
+        <v>94.80000000000001</v>
+      </c>
+      <c r="L5" t="n">
+        <v>89.54550634550634</v>
+      </c>
+      <c r="M5" t="n">
+        <v>-2.399999999999991</v>
+      </c>
+      <c r="N5" t="n">
+        <v>-0.8322751322751145</v>
+      </c>
+      <c r="O5" t="n">
+        <v>-2.400000000000006</v>
+      </c>
+      <c r="P5" t="n">
+        <v>-1.199999999999989</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>-2.42388722388722</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Detected_Action</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Random Forest</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>87.2</v>
+      </c>
+      <c r="D6" t="n">
+        <v>88.70952380952382</v>
+      </c>
+      <c r="E6" t="n">
+        <v>87.2</v>
+      </c>
+      <c r="F6" t="n">
+        <v>93.59999999999999</v>
+      </c>
+      <c r="G6" t="n">
+        <v>86.92155252155253</v>
+      </c>
+      <c r="H6" t="n">
+        <v>87.99999999999999</v>
+      </c>
+      <c r="I6" t="n">
+        <v>89.56507936507938</v>
+      </c>
+      <c r="J6" t="n">
+        <v>87.99999999999999</v>
+      </c>
+      <c r="K6" t="n">
+        <v>94.00000000000001</v>
+      </c>
+      <c r="L6" t="n">
+        <v>87.73872053872056</v>
+      </c>
+      <c r="M6" t="n">
+        <v>-0.7999999999999829</v>
+      </c>
+      <c r="N6" t="n">
+        <v>-0.8555555555555685</v>
+      </c>
+      <c r="O6" t="n">
+        <v>-0.7999999999999829</v>
+      </c>
+      <c r="P6" t="n">
+        <v>-0.4000000000000199</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>-0.8171680171680293</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Detected_Action</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>KNN</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>75.2</v>
+      </c>
+      <c r="D7" t="n">
+        <v>78.41428571428571</v>
+      </c>
+      <c r="E7" t="n">
+        <v>75.2</v>
+      </c>
+      <c r="F7" t="n">
+        <v>87.59999999999999</v>
+      </c>
+      <c r="G7" t="n">
+        <v>72.51971731971732</v>
+      </c>
+      <c r="H7" t="n">
+        <v>79.46666666666665</v>
+      </c>
+      <c r="I7" t="n">
+        <v>82.62962962962962</v>
+      </c>
+      <c r="J7" t="n">
+        <v>79.46666666666667</v>
+      </c>
+      <c r="K7" t="n">
+        <v>89.73333333333332</v>
+      </c>
+      <c r="L7" t="n">
+        <v>77.21881821881821</v>
+      </c>
+      <c r="M7" t="n">
+        <v>-4.266666666666652</v>
+      </c>
+      <c r="N7" t="n">
+        <v>-4.215343915343908</v>
+      </c>
+      <c r="O7" t="n">
+        <v>-4.266666666666666</v>
+      </c>
+      <c r="P7" t="n">
+        <v>-2.133333333333326</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>-4.699100899100898</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Detected_Action_Pipeline_PCA</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>SVM</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>92.8</v>
+      </c>
+      <c r="D8" t="n">
+        <v>94.17460317460318</v>
+      </c>
+      <c r="E8" t="n">
+        <v>92.8</v>
+      </c>
+      <c r="F8" t="n">
+        <v>96.40000000000001</v>
+      </c>
+      <c r="G8" t="n">
+        <v>92.71717171717169</v>
+      </c>
+      <c r="H8" t="n">
+        <v>89.59999999999998</v>
+      </c>
+      <c r="I8" t="n">
+        <v>91.96984126984125</v>
+      </c>
+      <c r="J8" t="n">
+        <v>89.59999999999999</v>
+      </c>
+      <c r="K8" t="n">
+        <v>94.80000000000001</v>
+      </c>
+      <c r="L8" t="n">
+        <v>89.54550634550634</v>
+      </c>
+      <c r="M8" t="n">
+        <v>3.200000000000017</v>
+      </c>
+      <c r="N8" t="n">
+        <v>2.204761904761924</v>
+      </c>
+      <c r="O8" t="n">
+        <v>3.200000000000003</v>
+      </c>
+      <c r="P8" t="n">
+        <v>1.599999999999994</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>3.171665371665355</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Detected_Action_Pipeline_PCA</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Random Forest</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>84.53333333333335</v>
+      </c>
+      <c r="D9" t="n">
+        <v>86.60634920634921</v>
+      </c>
+      <c r="E9" t="n">
+        <v>84.53333333333335</v>
+      </c>
+      <c r="F9" t="n">
+        <v>92.26666666666667</v>
+      </c>
+      <c r="G9" t="n">
+        <v>84.08620268620268</v>
+      </c>
+      <c r="H9" t="n">
+        <v>87.99999999999999</v>
+      </c>
+      <c r="I9" t="n">
+        <v>89.56507936507938</v>
+      </c>
+      <c r="J9" t="n">
+        <v>87.99999999999999</v>
+      </c>
+      <c r="K9" t="n">
+        <v>94.00000000000001</v>
+      </c>
+      <c r="L9" t="n">
+        <v>87.73872053872056</v>
+      </c>
+      <c r="M9" t="n">
+        <v>-3.46666666666664</v>
+      </c>
+      <c r="N9" t="n">
+        <v>-2.958730158730177</v>
+      </c>
+      <c r="O9" t="n">
+        <v>-3.46666666666664</v>
+      </c>
+      <c r="P9" t="n">
+        <v>-1.733333333333348</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>-3.652517852517875</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Detected_Action_Pipeline_PCA</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>KNN</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>72.26666666666667</v>
+      </c>
+      <c r="D10" t="n">
+        <v>75.06137566137566</v>
+      </c>
+      <c r="E10" t="n">
+        <v>72.26666666666667</v>
+      </c>
+      <c r="F10" t="n">
+        <v>86.13333333333334</v>
+      </c>
+      <c r="G10" t="n">
+        <v>68.8015984015984</v>
+      </c>
+      <c r="H10" t="n">
+        <v>79.46666666666665</v>
+      </c>
+      <c r="I10" t="n">
+        <v>82.62962962962962</v>
+      </c>
+      <c r="J10" t="n">
+        <v>79.46666666666667</v>
+      </c>
+      <c r="K10" t="n">
+        <v>89.73333333333332</v>
+      </c>
+      <c r="L10" t="n">
+        <v>77.21881821881821</v>
+      </c>
+      <c r="M10" t="n">
+        <v>-7.199999999999989</v>
+      </c>
+      <c r="N10" t="n">
+        <v>-7.568253968253956</v>
+      </c>
+      <c r="O10" t="n">
+        <v>-7.200000000000003</v>
+      </c>
+      <c r="P10" t="n">
+        <v>-3.59999999999998</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>-8.417219817219816</v>
       </c>
     </row>
   </sheetData>
@@ -1103,4 +1699,172 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Baseline</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Detected_Action</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Accuracy_Difference</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>KNN</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>79.46666666666665</v>
+      </c>
+      <c r="C2" t="n">
+        <v>75.2</v>
+      </c>
+      <c r="D2" t="n">
+        <v>-4.266666666666652</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SVM</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>89.59999999999998</v>
+      </c>
+      <c r="C3" t="n">
+        <v>87.19999999999999</v>
+      </c>
+      <c r="D3" t="n">
+        <v>-2.399999999999991</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Random Forest</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>87.99999999999999</v>
+      </c>
+      <c r="C4" t="n">
+        <v>87.2</v>
+      </c>
+      <c r="D4" t="n">
+        <v>-0.7999999999999829</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Baseline</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Detected_Action_Pipeline_PCA</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Accuracy_Difference</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>KNN</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>79.46666666666665</v>
+      </c>
+      <c r="C2" t="n">
+        <v>72.26666666666667</v>
+      </c>
+      <c r="D2" t="n">
+        <v>-7.199999999999989</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SVM</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>89.59999999999998</v>
+      </c>
+      <c r="C3" t="n">
+        <v>92.8</v>
+      </c>
+      <c r="D3" t="n">
+        <v>3.200000000000017</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Random Forest</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>87.99999999999999</v>
+      </c>
+      <c r="C4" t="n">
+        <v>84.53333333333335</v>
+      </c>
+      <c r="D4" t="n">
+        <v>-3.46666666666664</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>